<commit_message>
Update TA product backlog to version 2
</commit_message>
<xml_diff>
--- a/stage_1/product backlog template.xlsx
+++ b/stage_1/product backlog template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\10521\Desktop\软件工程\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenovo\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C7CCC75-2546-4232-95A2-51199F325659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7C6031B-CA22-48F5-BFF9-CE8FC972837C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -26,15 +26,12 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="109">
   <si>
     <t>Story ID</t>
   </si>
@@ -405,78 +402,16 @@
     <t>Supplementary function of account management, ensure system security, handle various account abnormal situations quickly</t>
   </si>
   <si>
-    <t>TA001</t>
-  </si>
-  <si>
-    <t>Comprehensive Personal Profile</t>
-  </si>
-  <si>
-    <t>1. Verify the system allows saving basic info, dynamically adding course records, and language scores.
-2. Verify the system prompts when mandatory fields are empty.
-3. Verify data is accurately written to a local data document.</t>
-  </si>
-  <si>
     <t>5 story points</t>
   </si>
   <si>
-    <t>Consolidates basic info, grades, language, and supplementary materials to streamline user input.</t>
-  </si>
-  <si>
-    <t>TA002</t>
-  </si>
-  <si>
-    <t>Submit CV</t>
-  </si>
-  <si>
-    <t>As a TA applicant, I want to upload my standardized CV in PDF format, so that the Module Organiser can comprehensively evaluate my overall academic abilities.</t>
-  </si>
-  <si>
     <t>Core strategy using internal file paths instead of external links.</t>
   </si>
   <si>
-    <t>TA003</t>
-  </si>
-  <si>
-    <t>Job Overview and Timetable(Optional)</t>
-  </si>
-  <si>
-    <t>As a TA applicant, I want to browse all open positions for the current semester and see the start dates and an optional timetable, so that I can understand job opportunities and judge time conflicts if the schedule is available.</t>
-  </si>
-  <si>
     <t>End dates of recruitment will be determined by MO; Timetable made optional as MOs cannot fully determine it before the semester.</t>
   </si>
   <si>
-    <t>TA004</t>
-  </si>
-  <si>
-    <t>Application Status Dashboard</t>
-  </si>
-  <si>
-    <t>As a TA applicant, I want to view the real-time review status of all historical applications in a dashboard, so that I can keep track of the progress at any time.</t>
-  </si>
-  <si>
-    <t>1. Verify historical applications are read and filtered by TA ID.
-2. Verify clear display of module, time, and status.
-3. Verify the frontend status updates synchronously with local data.</t>
-  </si>
-  <si>
     <t>Forms a closed loop of business flow on the TA side.</t>
-  </si>
-  <si>
-    <t>Lightweight implementation</t>
-  </si>
-  <si>
-    <t>Filtered by Start Date</t>
-  </si>
-  <si>
-    <t>As a TA applicant, I want to sort and filter open positions by their recruitment start date, so that I can prioritize applying for jobs that are starting soon.</t>
-  </si>
-  <si>
-    <t>1. Verify the system provides an option to sort the job list by start date(ascending/descending).
-2. Verify the sorted results accurately reflect the chronological order of the start dates.</t>
-  </si>
-  <si>
-    <t>Switched to sorting/filtering by start date based on the latest requirement.</t>
   </si>
   <si>
     <t>Filtered by Module Name</t>
@@ -585,51 +520,9 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>As a TA applicant, I want to create a comprehensive profile containing my basic personal info, undergraduate course grades, language proficiency and so on, so that the system can use it as a basic knowledge for TA application.</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>1. Verify the system provides a file upload mechanism restricted to PDF format.
 2. Verify this field is mandatory.
 3. Verify the system saves the files locally for displaying to MOs.</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Verify only current semester jobs are displayed.
-2. Verify clear display of MO, start dates, and timetable (if provided by MO).
-</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>Status Update Notice when login</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>As a TA applicant, I want the system to automatically present a notification upon login if there are status updates and new application statement feedback, so that I can be informed of the most important admission results immediately.</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>1. Verify the notice will always displays at the top of TA's homepage.
-2. Verify both TA's status and new application statement feedback can be viewed.
-3. Verify it will always displays when you go to TA's homepage.</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>TA009</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>Application Statement</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>As a TA applicant, I want to provide a dedicated application statement when applying for a specific TA position, so that I can have a further communication with the MO.</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Verify that a text box for writing the application statement appears during the application process.
-2. Verify that the application statement has a word limit and is an optional field.
-</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
@@ -678,6 +571,115 @@
 3. Job information is automatically saved as a JSON file after submission;
 4. Only the publishing MO can edit their own jobs, and administrators can view all MO-published jobs.
 5.MO can restrict only TA with specific conditions to apply at the time of release</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a TA applicant, I want to create a comprehensive profile containing my student ID, full name, email, phone number, research area and CET6 grade so that the system can use them as a basic knowledge for TA application.</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. Verify the system allows saving basic info, dynamically adding information.
+2. Verify the system prompts when mandatory fields are empty.
+3. Verify data is accurately written to a local data document.</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Record basic information of every TA and store them into system.</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>3 story points</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. Verify that the TA can select either the "leader" or "non-leader" role when submitting a course application.
+2. Verify that only three statuses are displayed in the application list: leader, non-leader, not hired.
+3. Verify that the role selected during application (leader / non-leader) is correctly stored and displayed in the application record.
+4. Verify that multiple TAs (including both leader and non-leader roles) can be admitted for a single course position simultaneously.</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>The same in the real world TA application.</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Should have</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Application Statement-Feedback Chat Box</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Submit CV</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>TA002</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>TA004</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Job Overview</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a TA applicant, I want to browse all the open jobs for the current semester and see the introduction of each job, so that I can decide which one to choose.</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Verify all the jobs are displayed.
+2. Verify clear display of MO, course name, introduction, requirements and timetable (if provided by MO).
+</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a TA applicant, I want to upload my CV in PDF format, so that the Module Organiser can comprehensively evaluate my overall academic abilities.</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>TA003</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>TA Application Role Selection</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a TA applicant, I want to be able to select to apply for either the leader or non-leader role when applying for a course position, so that I can clearly understand my application intention and admission result.</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a TA applicant, I want to view the real-time review status( "Approved as leader", "Approved as non-leader", or "reject") and feedback of all historical applications in a dashboard, so that I can keep track of the progress at any time.</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a TA applicant, I want to communicate with MD when apply for jobs, so that I can let MD have a better understanding of my overall abilities.</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. Verify that the chat box for typing words works during the application process.
+2. Verify that the chat box for typing words based on MD's feedback works at application status dashboard.                    3. Verify that there is a word limit in the chat box.</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Comprehensive Personal Profile</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>TA001</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Application Status Dashboard</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. Verify historical applications are read and filtered by TA ID.
+2. Verify clear display of module, time, and status and feedback.   3. Verify the frontend status updates synchronously with local data.                          4. Verify there is a note that exists when the status of one application changed.</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -796,9 +798,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 主题​​">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -836,9 +838,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -871,26 +873,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -923,26 +908,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1116,21 +1084,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J21"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
+  <dimension ref="A1:J20"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="16.625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="9.08984375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="16.6328125" style="1" customWidth="1"/>
     <col min="3" max="3" width="36" style="1" customWidth="1"/>
-    <col min="4" max="4" width="9.125" style="1"/>
-    <col min="5" max="5" width="28.375" style="1" customWidth="1"/>
-    <col min="6" max="7" width="19.875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="17.125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="24.875" style="1" customWidth="1"/>
-    <col min="10" max="10" width="26.375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="9.08984375" style="1"/>
+    <col min="5" max="5" width="28.36328125" style="1" customWidth="1"/>
+    <col min="6" max="7" width="19.90625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="17.08984375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="24.90625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="26.36328125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="27" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:10" ht="28" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1162,7 +1130,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="94.5" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:10" ht="98" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -1173,7 +1141,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="409.5" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:10" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>13</v>
       </c>
@@ -1184,7 +1152,7 @@
         <v>15</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>103</v>
+        <v>75</v>
       </c>
       <c r="E3" s="3">
         <v>1</v>
@@ -1205,7 +1173,7 @@
         <v>46107</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="375" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:10" ht="377" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>19</v>
       </c>
@@ -1216,7 +1184,7 @@
         <v>21</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>102</v>
+        <v>74</v>
       </c>
       <c r="E4" s="3">
         <v>1</v>
@@ -1237,9 +1205,9 @@
         <v>46132</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="225" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:10" ht="217.5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>107</v>
+        <v>79</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>25</v>
@@ -1248,7 +1216,7 @@
         <v>26</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>104</v>
+        <v>76</v>
       </c>
       <c r="E5" s="3">
         <v>1</v>
@@ -1269,9 +1237,9 @@
         <v>46112</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="330" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:10" ht="333.5" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>108</v>
+        <v>80</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>30</v>
@@ -1280,7 +1248,7 @@
         <v>31</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>104</v>
+        <v>76</v>
       </c>
       <c r="E6" s="3">
         <v>1</v>
@@ -1301,9 +1269,9 @@
         <v>46118</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="210" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:10" ht="217.5" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>109</v>
+        <v>81</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>34</v>
@@ -1312,7 +1280,7 @@
         <v>35</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>106</v>
+        <v>78</v>
       </c>
       <c r="E7" s="3">
         <v>1</v>
@@ -1333,30 +1301,30 @@
         <v>46124</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="180" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:10" ht="159.5" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E8" s="3">
+        <v>2</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="G8" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="E8" s="3">
-        <v>1</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>41</v>
-      </c>
       <c r="H8" s="3" t="s">
-        <v>42</v>
+        <v>86</v>
       </c>
       <c r="I8" s="5">
         <v>46101</v>
@@ -1365,30 +1333,30 @@
         <v>46107</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="135" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:10" ht="203" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>43</v>
+        <v>93</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>44</v>
+        <v>107</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>45</v>
+        <v>102</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>102</v>
+        <v>74</v>
       </c>
       <c r="E9" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>92</v>
+        <v>108</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>17</v>
+        <v>87</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="I9" s="5">
         <v>46101</v>
@@ -1397,30 +1365,30 @@
         <v>46107</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="120" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:10" ht="130.5" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>47</v>
+        <v>99</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>48</v>
+        <v>95</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>49</v>
+        <v>96</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>102</v>
+        <v>74</v>
       </c>
       <c r="E10" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="G10" s="3" t="s">
         <v>17</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="I10" s="5">
         <v>46101</v>
@@ -1429,30 +1397,30 @@
         <v>46107</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="150" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:10" ht="130.5" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>51</v>
+        <v>94</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>52</v>
+        <v>92</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>102</v>
+        <v>74</v>
       </c>
       <c r="E11" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>54</v>
+        <v>72</v>
       </c>
       <c r="G11" s="3" t="s">
         <v>17</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="I11" s="5">
         <v>46101</v>
@@ -1461,94 +1429,94 @@
         <v>46107</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="165" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:10" ht="362.5" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>87</v>
+        <v>68</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>102</v>
+        <v>75</v>
       </c>
       <c r="E12" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="G12" s="3" t="s">
         <v>24</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="I12" s="5">
-        <v>46113</v>
+        <v>46108</v>
       </c>
       <c r="J12" s="5">
-        <v>46119</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="150" x14ac:dyDescent="0.15">
+        <v>46112</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="188.5" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>88</v>
+        <v>69</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="D13" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="E13" s="3">
+        <v>2</v>
+      </c>
+      <c r="F13" s="3" t="s">
         <v>104</v>
-      </c>
-      <c r="E13" s="3">
-        <v>1</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>96</v>
       </c>
       <c r="G13" s="3" t="s">
         <v>24</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>56</v>
+        <v>73</v>
       </c>
       <c r="I13" s="5">
-        <v>46108</v>
+        <v>46113</v>
       </c>
       <c r="J13" s="5">
-        <v>46112</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="135" x14ac:dyDescent="0.15">
+        <v>46119</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="116" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>89</v>
+        <v>70</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>58</v>
+        <v>43</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>105</v>
+        <v>77</v>
       </c>
       <c r="E14" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="G14" s="3" t="s">
         <v>24</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="I14" s="5">
         <v>46113</v>
@@ -1557,30 +1525,30 @@
         <v>46119</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="120" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:10" ht="101.5" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>90</v>
+        <v>71</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>105</v>
+        <v>77</v>
       </c>
       <c r="E15" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="G15" s="3" t="s">
         <v>24</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="I15" s="5">
         <v>46113</v>
@@ -1589,62 +1557,62 @@
         <v>46119</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="90" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:10" ht="362.5" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>97</v>
+        <v>50</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>105</v>
+        <v>74</v>
       </c>
       <c r="E16" s="3">
         <v>1</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>67</v>
+        <v>83</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="I16" s="5">
-        <v>46113</v>
+        <v>46101</v>
       </c>
       <c r="J16" s="5">
-        <v>46119</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="330" x14ac:dyDescent="0.15">
+        <v>46107</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="290" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>71</v>
+        <v>56</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>102</v>
+        <v>74</v>
       </c>
       <c r="E17" s="3">
         <v>1</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>111</v>
+        <v>82</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>72</v>
+        <v>57</v>
       </c>
       <c r="I17" s="5">
         <v>46101</v>
@@ -1653,30 +1621,30 @@
         <v>46107</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="270" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:10" ht="304.5" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="B18" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D18" s="3" t="s">
         <v>74</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>102</v>
       </c>
       <c r="E18" s="3">
         <v>1</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>110</v>
+        <v>61</v>
       </c>
       <c r="G18" s="3" t="s">
         <v>24</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>76</v>
+        <v>62</v>
       </c>
       <c r="I18" s="5">
         <v>46101</v>
@@ -1685,81 +1653,49 @@
         <v>46107</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="300" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:10" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>102</v>
+        <v>76</v>
       </c>
       <c r="E19" s="3">
         <v>1</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>80</v>
+        <v>66</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="I19" s="5">
-        <v>46101</v>
+        <v>46108</v>
       </c>
       <c r="J19" s="5">
-        <v>46107</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="390" x14ac:dyDescent="0.15">
-      <c r="A20" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="E20" s="3">
-        <v>1</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H20" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="I20" s="5">
-        <v>46108</v>
-      </c>
-      <c r="J20" s="5">
         <v>46112</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="15" x14ac:dyDescent="0.15">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="3"/>
-      <c r="H21" s="3"/>
-      <c r="I21" s="5"/>
-      <c r="J21" s="5"/>
+    <row r="20" spans="1:10" ht="14.5" x14ac:dyDescent="0.25">
+      <c r="A20" s="3"/>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
"Update some functions of TA"
</commit_message>
<xml_diff>
--- a/stage_1/product backlog template.xlsx
+++ b/stage_1/product backlog template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenovo\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\software_engineering\software-engineering\stage_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7C6031B-CA22-48F5-BFF9-CE8FC972837C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{161E099C-428E-459C-B2EC-2B28C786AA14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -414,9 +414,6 @@
     <t>Forms a closed loop of business flow on the TA side.</t>
   </si>
   <si>
-    <t>Filtered by Module Name</t>
-  </si>
-  <si>
     <t>As a TA applicant, I want to search the current job list by entering a "module name", so that I can quickly locate courses relevant to my major.</t>
   </si>
   <si>
@@ -653,10 +650,6 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>As a TA applicant, I want to view the real-time review status( "Approved as leader", "Approved as non-leader", or "reject") and feedback of all historical applications in a dashboard, so that I can keep track of the progress at any time.</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>As a TA applicant, I want to communicate with MD when apply for jobs, so that I can let MD have a better understanding of my overall abilities.</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -680,6 +673,14 @@
   <si>
     <t>1. Verify historical applications are read and filtered by TA ID.
 2. Verify clear display of module, time, and status and feedback.   3. Verify the frontend status updates synchronously with local data.                          4. Verify there is a note that exists when the status of one application changed.</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a TA applicant, I want to view the real-time review status( "Approved as leader", "Approved as non-leader", "reject" or "interviewed") and feedback of all historical applications in a dashboard, so that I can keep track of the progress at any time.</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Search for Module Name</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -1152,7 +1153,7 @@
         <v>15</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E3" s="3">
         <v>1</v>
@@ -1184,7 +1185,7 @@
         <v>21</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E4" s="3">
         <v>1</v>
@@ -1207,7 +1208,7 @@
     </row>
     <row r="5" spans="1:10" ht="217.5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>25</v>
@@ -1216,7 +1217,7 @@
         <v>26</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E5" s="3">
         <v>1</v>
@@ -1239,7 +1240,7 @@
     </row>
     <row r="6" spans="1:10" ht="333.5" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>30</v>
@@ -1248,7 +1249,7 @@
         <v>31</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E6" s="3">
         <v>1</v>
@@ -1271,7 +1272,7 @@
     </row>
     <row r="7" spans="1:10" ht="217.5" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>34</v>
@@ -1280,7 +1281,7 @@
         <v>35</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E7" s="3">
         <v>1</v>
@@ -1303,28 +1304,28 @@
     </row>
     <row r="8" spans="1:10" ht="159.5" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E8" s="3">
         <v>2</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G8" s="3" t="s">
         <v>38</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="I8" s="5">
         <v>46101</v>
@@ -1335,25 +1336,25 @@
     </row>
     <row r="9" spans="1:10" ht="203" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B9" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>102</v>
-      </c>
       <c r="D9" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E9" s="3">
         <v>2</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H9" s="3" t="s">
         <v>41</v>
@@ -1367,22 +1368,22 @@
     </row>
     <row r="10" spans="1:10" ht="130.5" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B10" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>96</v>
-      </c>
       <c r="D10" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E10" s="3">
         <v>2</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G10" s="3" t="s">
         <v>17</v>
@@ -1399,22 +1400,22 @@
     </row>
     <row r="11" spans="1:10" ht="130.5" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E11" s="3">
         <v>2</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G11" s="3" t="s">
         <v>17</v>
@@ -1431,28 +1432,28 @@
     </row>
     <row r="12" spans="1:10" ht="362.5" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B12" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="C12" s="3" t="s">
-        <v>101</v>
-      </c>
       <c r="D12" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E12" s="3">
         <v>2</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G12" s="3" t="s">
         <v>24</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="I12" s="5">
         <v>46108</v>
@@ -1463,28 +1464,28 @@
     </row>
     <row r="13" spans="1:10" ht="188.5" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E13" s="3">
         <v>2</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="G13" s="3" t="s">
         <v>24</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I13" s="5">
         <v>46113</v>
@@ -1495,28 +1496,28 @@
     </row>
     <row r="14" spans="1:10" ht="116" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B14" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C14" s="3" t="s">
-        <v>43</v>
-      </c>
       <c r="D14" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E14" s="3">
         <v>2</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G14" s="3" t="s">
         <v>24</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I14" s="5">
         <v>46113</v>
@@ -1527,28 +1528,28 @@
     </row>
     <row r="15" spans="1:10" ht="101.5" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B15" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C15" s="3" t="s">
-        <v>47</v>
-      </c>
       <c r="D15" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E15" s="3">
         <v>2</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G15" s="3" t="s">
         <v>24</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I15" s="5">
         <v>46113</v>
@@ -1559,28 +1560,28 @@
     </row>
     <row r="16" spans="1:10" ht="362.5" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="C16" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="C16" s="3" t="s">
-        <v>52</v>
-      </c>
       <c r="D16" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E16" s="3">
         <v>1</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G16" s="3" t="s">
         <v>17</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I16" s="5">
         <v>46101</v>
@@ -1591,28 +1592,28 @@
     </row>
     <row r="17" spans="1:10" ht="290" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="C17" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="C17" s="3" t="s">
-        <v>56</v>
-      </c>
       <c r="D17" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E17" s="3">
         <v>1</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G17" s="3" t="s">
         <v>24</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="I17" s="5">
         <v>46101</v>
@@ -1623,28 +1624,28 @@
     </row>
     <row r="18" spans="1:10" ht="304.5" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="C18" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C18" s="3" t="s">
-        <v>60</v>
-      </c>
       <c r="D18" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E18" s="3">
         <v>1</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G18" s="3" t="s">
         <v>24</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I18" s="5">
         <v>46101</v>
@@ -1655,28 +1656,28 @@
     </row>
     <row r="19" spans="1:10" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="C19" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="C19" s="3" t="s">
-        <v>65</v>
-      </c>
       <c r="D19" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E19" s="3">
         <v>1</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G19" s="3" t="s">
         <v>17</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I19" s="5">
         <v>46108</v>

</xml_diff>